<commit_message>
feat: incremento 6 (cronograma estimado, tarefas por pavimento e WhatsApp no computador)
- estimativa automática do §13: prazo sugerido pela área, pavimentos e estrutura;
  etapas típicas com sobreposição; bloco estrutural por pavimento; selo ESTIMATIVA
  e aviso no relatório; substituição com confirmação
- campo pavimento nas tarefas (CSV, XLSX, JSON, editor, exportações e modelos):
  limita as regras ao pavimento, então no sobrado as paredes de cima esperam a laje
- 'Enviar pelo WhatsApp' quando não há Web Share de arquivos: baixa o vídeo e abre
  o WhatsApp Web; 'Compartilhar…' segue nos aparelhos que permitem
- corrige laço infinito do React (seletor que criava lista nova a cada leitura)
- ADR-18, ADR-19 e ADR-20; 10 testes Vitest e 3 Playwright novos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelos/cronograma-modelo.xlsx
+++ b/public/modelos/cronograma-modelo.xlsx
@@ -401,16 +401,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:I16"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="8.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,12 +431,15 @@
         <v>categoria</v>
       </c>
       <c r="F1" t="str">
+        <v>pavimento</v>
+      </c>
+      <c r="G1" t="str">
         <v>inicio_real</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>fim_real</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>avanco</v>
       </c>
     </row>
@@ -455,13 +459,13 @@
       <c r="E2" t="str">
         <v>terreno</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>46027</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>46037</v>
       </c>
-      <c r="H2" s="2">
+      <c r="I2" s="2">
         <v>1</v>
       </c>
     </row>
@@ -481,13 +485,13 @@
       <c r="E3" t="str">
         <v>fundacao</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="1">
         <v>46038</v>
       </c>
-      <c r="G3" s="1">
+      <c r="H3" s="1">
         <v>46061</v>
       </c>
-      <c r="H3" s="2">
+      <c r="I3" s="2">
         <v>1</v>
       </c>
     </row>
@@ -507,13 +511,13 @@
       <c r="E4" t="str">
         <v>estrutura</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>46062</v>
       </c>
-      <c r="G4" s="1">
+      <c r="H4" s="1">
         <v>46087</v>
       </c>
-      <c r="H4" s="2">
+      <c r="I4" s="2">
         <v>1</v>
       </c>
     </row>
@@ -533,13 +537,13 @@
       <c r="E5" t="str">
         <v>alvenaria</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="1">
         <v>46088</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>46122</v>
       </c>
-      <c r="H5" s="2">
+      <c r="I5" s="2">
         <v>1</v>
       </c>
     </row>
@@ -559,10 +563,10 @@
       <c r="E6" t="str">
         <v>laje</v>
       </c>
-      <c r="F6" s="1">
+      <c r="G6" s="1">
         <v>46123</v>
       </c>
-      <c r="H6" s="2">
+      <c r="I6" s="2">
         <v>0.6</v>
       </c>
     </row>
@@ -599,10 +603,10 @@
       <c r="E8" t="str">
         <v>instalacoes</v>
       </c>
-      <c r="F8" s="1">
+      <c r="G8" s="1">
         <v>46130</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I8" s="2">
         <v>0.15</v>
       </c>
     </row>
@@ -744,14 +748,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -831,115 +835,126 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>inicio_real</v>
+        <v>pavimento</v>
       </c>
       <c r="B9" t="str">
         <v>não</v>
       </c>
       <c r="C9" t="str">
-        <v>Data em que a tarefa começou de fato</v>
+        <v>Limita a tarefa aos elementos de um pavimento (ex.: Térreo); em branco, vale para o prédio inteiro</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>fim_real</v>
+        <v>inicio_real</v>
       </c>
       <c r="B10" t="str">
         <v>não</v>
       </c>
       <c r="C10" t="str">
-        <v>Data em que terminou de fato (exige inicio_real)</v>
+        <v>Data em que a tarefa começou de fato</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>avanco</v>
+        <v>fim_real</v>
       </c>
       <c r="B11" t="str">
         <v>não</v>
       </c>
       <c r="C11" t="str">
+        <v>Data em que terminou de fato (exige inicio_real)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>avanco</v>
+      </c>
+      <c r="B12" t="str">
+        <v>não</v>
+      </c>
+      <c r="C12" t="str">
         <v>Avanço físico medido: 0% a 100%; vazio = deduzido das datas reais</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Categorias com regra automática</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>terreno</v>
+        <v>Categorias com regra automática</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>fundacao</v>
+        <v>terreno</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>estrutura</v>
+        <v>fundacao</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>alvenaria</v>
+        <v>estrutura</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>laje</v>
+        <v>alvenaria</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>cobertura</v>
+        <v>laje</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>instalacoes</v>
+        <v>cobertura</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>reboco</v>
+        <v>instalacoes</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>esquadrias</v>
+        <v>reboco</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>revestimento</v>
+        <v>esquadrias</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>pintura</v>
+        <v>revestimento</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>loucas</v>
+        <v>pintura</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>loucas</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>paisagismo</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="str">
+    <row r="29">
+      <c r="A29" t="str">
         <v>O app lê só a primeira planilha (Cronograma). Os dados deste modelo são fictícios.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>